<commit_message>
feat: inital extraction to
</commit_message>
<xml_diff>
--- a/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
+++ b/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
@@ -5,16 +5,20 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data\luat_dat_dai\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\LawAssistant\triplet_extraction\data\luat_dat_dai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CCB54C-252C-4818-9AFA-81265B50B531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF4D1A1-B0B6-4E79-84FA-DEAAAB81A366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75A87B30-D479-4520-B3E8-6EE7229C7E16}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="loai_1" localSheetId="0">Sheet1!$B$4</definedName>
+    <definedName name="loai_1_name" localSheetId="0">Sheet1!$B$5</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="199">
   <si>
     <t>31/2024/QH15</t>
   </si>
@@ -218,9 +222,6 @@
     <t>56/2024/TT-BCA</t>
   </si>
   <si>
-    <t xml:space="preserve"> so_hieu</t>
-  </si>
-  <si>
     <t>VanBanGoc_31-2024-qh15_1.pdf</t>
   </si>
   <si>
@@ -248,9 +249,6 @@
     <t>23.2003.QH11.doc</t>
   </si>
   <si>
-    <t>VanBanGoc_2024_987 + 988_43-2024-QH15..pdf</t>
-  </si>
-  <si>
     <t>VanBanGoc_59.signed.pdf</t>
   </si>
   <si>
@@ -398,9 +396,6 @@
     <t>50-btnmt.pdf</t>
   </si>
   <si>
-    <t>TT29-2024-TT-BTNMT_Signed-quyđịnhkỹthuậtlập</t>
-  </si>
-  <si>
     <t>11-bnv.pdf</t>
   </si>
   <si>
@@ -444,13 +439,302 @@
   </si>
   <si>
     <t>title</t>
+  </si>
+  <si>
+    <t>Luật Đất đai</t>
+  </si>
+  <si>
+    <t>NGHỊ QUYẾT
+VỀ NHÀ ĐẤT DO NHÀ NƯỚC ĐÃ QUẢN LÝ, BỐ TRÍ SỬ DỤNG TRONG QUÁ TRÌNH THỰC HIỆN CÁC CHÍNH SÁCH QUẢN LÝ NHÀ ĐẤT VÀ CHÍNH SÁCH CẢI TẠO XÃ HỘI CHỦ NGHĨA TRƯỚC NGÀY 01 THÁNG 7 NĂM 1991</t>
+  </si>
+  <si>
+    <t>LUẬT
+SỬA ĐỔI, BỔ SUNG MỘT SỐ ĐIỀU
+CỦA LUẬT ĐẤT ĐAI SỐ 31/2024/QH15, LUẬT NHÀ Ở SỐ 27/2023/QH15,
+LUẬT KINH DOANH BẤT ĐỘNG SẢN SỐ 29/2023/QH15 VÀ
+LUẬT CÁC TỔ CHỨC TÍN DỤNG SỐ 32/2024/QH15</t>
+  </si>
+  <si>
+    <t>Luật doanh nghiệp</t>
+  </si>
+  <si>
+    <t>LUẬT 
+SỬA ĐỔI, BỔ SUNG MỘT SỐ ĐIỀU CỦA LUẬT QUY HOẠCH,          LUẬT ĐẦU TƯ, LUẬT ĐẦU TƯ THEO PHƯƠNG THỨC ĐỐI TÁC CÔNG TƯ VÀ LUẬT ĐẤU THẦU</t>
+  </si>
+  <si>
+    <t>LUẬT
+QUY HOẠCH</t>
+  </si>
+  <si>
+    <t>Luật đầu tư</t>
+  </si>
+  <si>
+    <t>LUẬT
+ĐẦU TƯ CÔNG</t>
+  </si>
+  <si>
+    <t>LUẬT
+SỬA ĐỔI, BỔ SUNG MỘT SỐ ĐIỀU CỦA LUẬT ĐẤU THẦU, LUẬT
+ĐẦU TƯ THEO PHƯƠNG THỨC ĐỐI TÁC CÔNG TƯ, LUẬT HẢI
+QUAN, LUẬT THUẾ GIÁ TRỊ GIA TĂNG, LUẬT THUẾ XUẤT KHẨU,
+THUẾ NHẬP KHẨU, LUẬT ĐẦU TƯ, LUẬT ĐẦU TƯ CÔNG, LUẬT
+QUẢN LÝ, SỬ DỤNG TÀI SẢN CÔNG</t>
+  </si>
+  <si>
+    <t>Luật kiến trúc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUẬT
+Hôn nhân và gia đình </t>
+  </si>
+  <si>
+    <t>LUẬT
+NHÀ Ở</t>
+  </si>
+  <si>
+    <t>LUẬT
+THUẾ SỬ DỤNG ĐẤT PHI NÔNG NGHIỆP</t>
+  </si>
+  <si>
+    <t>LUẬT
+Của Quốc hội nước Cộng hoà xã hội chủ nghĩa Việt Nam số 17-1999/QH10 về sửa đổi, bổ sung một số điều của Luật thuế chuyển quyền sử dụng đất</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Sửa đổi, bổ sung một số điều của Nghị định số 100/2024/NĐ-CP ngày 26 tháng 7 năm 2024 của Chính phủ quy định chi tiết một số điều của Luật Nhà ở về phát triển và quản lý nhà ở xã hội và Nghị định số 192/2025/NĐ-CP ngày 01 tháng 7 năm 2025 của Chính phủ quy định chi tiết một số điều và biện pháp thi hành Nghị quyết số 201/2025/QH15 ngày 29 tháng 5 năm 2025 của Quốc hội thí điểm về một số cơ chế, chính sách đặc thù phát triển nhà ở xã hội</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Về quản lý công viên, cây xanh, mặt nước</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định các trường hợp khác được miễn, giảm tiền sử dụng đất,
+tiền thuê đất theo quy định tại khoản 2 Điều 157 Luật Đất đai năm 2024</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+SỬA ĐỔI, BỔ SUNG MỘT SỐ ĐIỀU CỦA CÁC NGHỊ ĐỊNH QUY ĐỊNH CHI TIẾT THI HÀNH LUẬT ĐẤT ĐAI</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định chi tiết một số điều và biện pháp thi hành Nghị quyết
+số 201/2025/QH15 ngày 29 tháng 5 năm 2025 của Quốc hội thí điểm
+về một số cơ chế, chính sách đặc thù phát triển nhà ở xã hội</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định chi tiết thi hành Nghị quyết số 171/2024/QH15 ngày 30 tháng 11
+năm 2024 của Quốc hội về thí điểm thực hiện dự án nhà ở thương mại thông
+qua thỏa thuận về nhận quyền sử dụng đất hoặc đang có quyền sử dụng đất</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về giá đất</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về phân định thẩm quyền của chính quyền địa phương 02 cấp,
+phân quyền, phân cấp trong lĩnh vực đất đai</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về phân quyền, phân cấp trong                                                              lĩnh vực quản lý nhà nước của Bộ Xây dựng</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định phân định thẩm quyền của chính quyền địa phương 02 cấp
+trong lĩnh vực quản lý nhà nước của Bộ Nông nghiệp và Môi trường</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định chi tiết một số điều của Luật Quy hoạch đô thị và nông thôn</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về phân định thẩm quyền của chính quyền địa phương
+02 cấp trong lĩnh vực quản lý nhà nước của Bộ Xây dựng</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về xử phạt vi phạm hành chính trong lĩnh vực đất đai</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định chi tiết một số điều và biện pháp thi hành Luật Đấu thầu về lựa chọn nhà đầu tư thực hiện dự án đầu tư có sử dụng đất</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định việc quản lý, sử dụng và khai thác nhà, đất là tài sản công
+không sử dụng vào mục đích để ở giao cho tổ chức có chức năng quản lý,
+kinh doanh nhà địa phương quản lý, khai thác</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về Quỹ phát triển đất</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về tiền sử dụng đất, tiền thuê đất</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định chi tiết thi hành một số điều của Luật Đất đai</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về điều tra cơ bản đất đai; đăng ký, cấp Giấy chứng nhận 
+quyền sử dụng đất, quyền sở hữu tài sản gắn liền với đất 
+và Hệ thống thông tin đất đai</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định chi tiết một số điều của Luật Nhà ở 
+về phát triển và quản lý nhà ở xã hội</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định chi tiết một số điều của Luật Nhà ở 
+về cải tạo, xây dựng lại nhà chung cư</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NGHỊ ĐỊNH
+Quy định chi tiết một số điều của Luật Kinh doanh bất động sản </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NGHỊ ĐỊNH
+Quy định chi tiết một số điều của Luật Nhà ở </t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định chi tiết một số điều của Luật Kinh doanh bất động sản
+vệ xây dựng và quản lý hệ thống thông tin, cơ sở dữ liệu về nhà ở và thị trường bất động sản</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định việc giảm tiền thuê đất năm 2024</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH 
+Quy định về bồi thường, hỗ trợ, tái định cư khi Nhà nước thu hồi đất</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Sửa đổi, bổ sung một số điều của các Nghị định hướng dẫn thi hành Luật Đất đai</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Về xây dựng, quản lý và sử dụng hệ thống thông tin
+về nhà ở và thị trường bất động sản</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định về khung giá đất</t>
+  </si>
+  <si>
+    <t>QUYẾT ĐỊNH
+VỀ CƠ CHẾ, CHÍNH SÁCH GIẢI QUYẾT VIỆC LÀM VÀ ĐÀO TẠO NGHỀ CHO NGƯỜI CÓ ĐẤT THU HỒI</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Quy định định mức kinh tế - kỹ thuật
+thống kê, kiểm kê đất đai, lập bản đồ hiện trạng sử dụng đất và xây dựng
+cơ sở dữ liệu quốc gia về đất đai</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Quy định định mức kinh tế - kỹ thuật điều tra, đánh giá đất đai
+cấp vùng và cả nước</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THÔNG TƯ
+Quy định kỹ thuật về lập, điều chỉnh quy hoạch, kế hoạch sử dụng đất </t>
+  </si>
+  <si>
+    <t>TT29-2024-TT-BTNMT_Signed-quyđịnhkỹthuậtlập.doc</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Quy định về việc lập, quản lý hồ sơ địa giới đơn vị hành chính</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Quy định mức thu, chế độ thu, nộp, quản lý,
+sử dụng phí khai thác và sử dụng tài liệu đất đai từ
+Hệ thống thông tin quốc gia về đất đai</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Quy định về hồ sơ địa chính, Giấy chứng nhận
+quyền sử dụng đất, quyền sở hữu tài sản gắn liền với đất</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Quy định phân cấp, phân định thẩm quyền quản lý nhà nước
+trong lĩnh vực đất đai</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Sửa đổi, bổ sung, bãi bỏ các Thông tư của Bộ trưởng Bộ Tài chính trong lĩnh
+vực kế toán, kiểm toán để đẩy mạnh phân cấp, phân quyền và sắp xếp tổ chức
+chính quyền địa phương 02 cấp</t>
+  </si>
+  <si>
+    <t>NGHỊ QUYẾT
+Quy định việc giải quyết đối với một số trường hợp cụ thể về nhà đất 
+trong quá trình thực hiện các chính sách quản lý nhà đất và chính sách cải tạo xã hội chủ nghĩa trước ngày 01 tháng 07 năm 1991</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Hướng dẫn về chương trình khung đào tạo, bồi dưỡng kiến thức hành nghề
+môi giới bất động sản, điều hành sàn giao dịch bất động sản</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Hướng dẫn sử dung kinh phí xay dung, quản lý, van hanh va khai thác hệ
+thống thông tin, cơ sở dữ liệu về nhà ở và thị trường bất động sản</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THÔNG TƯ
+Quy định chi tiết một số điều của Luật Nhà ở </t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Sửa đổi, bổ sung một số điều của các Thông tư thuộc lĩnh vực quản lý nhà nước của Bộ Xây dựng liên quan đến sắp xếp tổ chức bộ máy, thực hiện chính quyền địa phương 02 cấp và phân cấp cho chính quyền địa phương</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+Quy định chi tiết một số điều của Luật Nhà ở trong Công an nhân dân</t>
+  </si>
+  <si>
+    <t>THÔNG TƯ
+QUY ĐỊNH CHI TIẾT MỘT SỐ ĐIỀU CỦA LUẬT NHÀ Ở TRONG QUÂN ĐỘI NHÂN DÂN VIỆT NAM</t>
+  </si>
+  <si>
+    <t>effective date</t>
+  </si>
+  <si>
+    <t> 29/11/2024</t>
+  </si>
+  <si>
+    <t>Luật Dân sự</t>
+  </si>
+  <si>
+    <t>LUẬT 
+KINH DOANH BẤT ĐỘNG SẢN</t>
+  </si>
+  <si>
+    <t>VanBanGoc_2024_987 + 988_43-2024-QH15.pdf</t>
+  </si>
+  <si>
+    <t>so_hieu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -460,6 +744,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -485,13 +776,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -827,555 +1142,939 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED14D7C1-14A4-44A5-A6EE-F18154C6E1E7}">
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22" style="2" customWidth="1"/>
-    <col min="3" max="5" width="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28" style="10" customWidth="1"/>
+    <col min="4" max="4" width="29.5546875" style="3" customWidth="1"/>
+    <col min="5" max="6" width="28" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C1" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B2" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C2" s="7">
+        <v>45309</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s">
         <v>61</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>62</v>
       </c>
-      <c r="E2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B3" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C3" s="7">
+        <v>42332</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" t="s">
         <v>64</v>
       </c>
-      <c r="D3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B4" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" s="7">
+        <v>37951</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" s="7">
+        <v>45472</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B6" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" s="7">
+        <v>43999</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="C7" s="7">
+        <v>45258</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B8" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C8" s="7">
+        <v>45625</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C9" s="7">
+        <v>43063</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B10" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10" s="7">
+        <v>43999</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B11" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B12" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C12" s="7">
+        <v>45833</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C13" s="7">
+        <v>43629</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C14" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C14" s="7">
+        <v>41809</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C15" t="s">
-        <v>81</v>
-      </c>
-      <c r="D15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C15" s="7">
+        <v>45257</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C16" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C16" s="7">
+        <v>40348</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C17" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C17" s="7">
+        <v>36515</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="216" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C18" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B18" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="7">
+        <v>45940</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C19" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B19" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C19" s="7">
+        <v>45939</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C20" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B20" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C20" s="9">
+        <v>45888</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C21" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B21" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C21" s="7">
+        <v>45884</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C22" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B22" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C22" s="7">
+        <v>45839</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="144" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C23" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B23" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C23" s="7">
+        <v>45748</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C24" t="s">
-        <v>91</v>
-      </c>
-      <c r="D24" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B24" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C24" s="7">
+        <v>45470</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E24" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B25" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" s="7">
+        <v>45820</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C26" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B26" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C26" s="7">
+        <v>45820</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C27" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B27" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C27" s="7">
+        <v>45820</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C28" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B28" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C28" s="9">
+        <v>45658</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C29" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B29" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C29" s="9">
+        <v>45839</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C30" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B30" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C30" s="9">
+        <v>45820</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C31" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B31" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" s="7">
+        <v>45569</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="72" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C32" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B32" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C32" s="7">
+        <v>45551</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C33" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B33" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C33" s="7">
+        <v>45527</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C34" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B34" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C34" s="7">
+        <v>45504</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C35" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B35" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="C35" s="7">
+        <v>45503</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C36" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B36" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C36" s="7">
+        <v>45503</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C37" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B37" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C37" s="7">
+        <v>45502</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C38" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B38" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C38" s="7">
+        <v>45499</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C39" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B39" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C39" s="7">
+        <v>45498</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C40" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B40" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C40" s="7">
+        <v>45497</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C41" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B41" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C41" s="7">
+        <v>45257</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C42" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B42" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C42" s="7">
+        <v>45497</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C43" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B43" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C43" s="7">
+        <v>45758</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C44" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B44" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C44" s="7">
+        <v>45488</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C45" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B45" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C45" s="7">
+        <v>45470</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C46" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B46" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C46" s="7">
+        <v>45019</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C47" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B47" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C47" s="7">
+        <v>44741</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C48" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B48" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C48" s="7">
+        <v>43818</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C49" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B49" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="C49" s="7">
+        <v>45504</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C50" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B50" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C50" s="7">
+        <v>45657</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C51" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B51" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C51" s="7">
+        <v>45657</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C52" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B52" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C52" s="7">
+        <v>45638</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C53" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B53" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C53" s="7">
+        <v>45583</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C54" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B54" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C54" s="7">
+        <v>45504</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C55" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B55" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C55" s="7">
+        <v>45504</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C56" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C56" s="7">
+        <v>45828</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C57" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B57" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C57" s="7">
+        <v>45828</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C58" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B58" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C58" s="9">
+        <v>38444</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C59" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B59" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="C59" s="7">
+        <v>45503</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C60" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B60" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C60" s="7">
+        <v>45621</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C61" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B61" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C61" s="7">
+        <v>45504</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C62" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B62" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C62" s="7">
+        <v>45821</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C63" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B63" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C63" s="7">
+        <v>45601</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C64" t="s">
-        <v>134</v>
+        <v>130</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C64" s="7">
+        <v>45607</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: finish extracting text from data
</commit_message>
<xml_diff>
--- a/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
+++ b/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\LawAssistant\triplet_extraction\data\luat_dat_dai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF4D1A1-B0B6-4E79-84FA-DEAAAB81A366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D095DC19-247F-4E0F-B2BE-B791DE83AA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75A87B30-D479-4520-B3E8-6EE7229C7E16}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="198">
   <si>
     <t>31/2024/QH15</t>
   </si>
@@ -712,9 +712,6 @@
   </si>
   <si>
     <t>effective date</t>
-  </si>
-  <si>
-    <t> 29/11/2024</t>
   </si>
   <si>
     <t>Luật Dân sự</t>
@@ -776,7 +773,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -797,9 +794,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1147,14 +1141,14 @@
   <cols>
     <col min="1" max="1" width="22" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28" style="10" customWidth="1"/>
+    <col min="3" max="3" width="28" style="9" customWidth="1"/>
     <col min="4" max="4" width="29.5546875" style="3" customWidth="1"/>
     <col min="5" max="6" width="28" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>132</v>
@@ -1197,7 +1191,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C3" s="7">
         <v>42332</v>
@@ -1234,7 +1228,7 @@
         <v>45472</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -1259,7 +1253,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C7" s="7">
         <v>45258</v>
@@ -1317,8 +1311,8 @@
       <c r="B11" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>194</v>
+      <c r="C11" s="7">
+        <v>45625</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>75</v>
@@ -1446,7 +1440,7 @@
       <c r="B20" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>45888</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -1561,7 +1555,7 @@
       <c r="B28" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="C28" s="9">
+      <c r="C28" s="8">
         <v>45658</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -1575,7 +1569,7 @@
       <c r="B29" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="C29" s="9">
+      <c r="C29" s="8">
         <v>45839</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -1589,7 +1583,7 @@
       <c r="B30" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C30" s="9">
+      <c r="C30" s="8">
         <v>45820</v>
       </c>
       <c r="D30" s="3" t="s">
@@ -1981,7 +1975,7 @@
       <c r="B58" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C58" s="9">
+      <c r="C58" s="8">
         <v>38444</v>
       </c>
       <c r="D58" s="3" t="s">

</xml_diff>

<commit_message>
feat: fix error in document extraction and remove docx data
</commit_message>
<xml_diff>
--- a/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
+++ b/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\LawAssistant\triplet_extraction\data\luat_dat_dai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D095DC19-247F-4E0F-B2BE-B791DE83AA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471DD5CE-8481-49CF-A714-496FDDA5FC46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75A87B30-D479-4520-B3E8-6EE7229C7E16}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
   <si>
     <t>31/2024/QH15</t>
   </si>
@@ -294,30 +294,18 @@
     <t>261_2025_ND-CP_661849.doc</t>
   </si>
   <si>
-    <t>258_2025_ND-CP_09102025.docx</t>
-  </si>
-  <si>
     <t>VanBanGoc_230.NĐ.pdf</t>
   </si>
   <si>
     <t>226_2025_ND-CP_664033.doc</t>
   </si>
   <si>
-    <t>Nghịđịnh-192-2025-NĐ-CP.docx</t>
-  </si>
-  <si>
-    <t>VanBanGoc_2025_629 + 630_75-2025-NĐ-CP..pdf</t>
-  </si>
-  <si>
     <t>VanBanGoc_ND 71-2024-ND-CP_01.pdf</t>
   </si>
   <si>
     <t>VanBanGoc_ND 71-2024-ND-CP_02.pdf</t>
   </si>
   <si>
-    <t>VanBanGoc_Nghị định-151-2025-NĐ-CP Nghị định 1512025NĐ-CP về thẩm quyền chính quyền địa phương 02 cấp trong đất đai-đã nén-trang-1.pdf</t>
-  </si>
-  <si>
     <t>Nghịđịnh144.2025.NĐ-CP.doc</t>
   </si>
   <si>
@@ -327,57 +315,18 @@
     <t>VanBanGoc_03.pdf</t>
   </si>
   <si>
-    <t>Nghịđịnh178.2025.NĐ-CP.docx</t>
-  </si>
-  <si>
-    <t>Nghịđịnh-140-2025-NĐ-CP.docx</t>
-  </si>
-  <si>
     <t>VanBanGoc_123-2024-nđ-cp.pdf</t>
   </si>
   <si>
-    <t>115.2024.NĐ.CP(W).docx</t>
-  </si>
-  <si>
-    <t>VanBanGoc_108-đã nén.pdf</t>
-  </si>
-  <si>
     <t>VanBanGoc_104.pdf</t>
   </si>
   <si>
-    <t>VanBanGoc_103-nd.signed.pdf</t>
-  </si>
-  <si>
     <t>Nghịđịnh102.2024.NĐ.CP.doc</t>
   </si>
   <si>
-    <t>NĐ100.2024.NĐ.CP.docx</t>
-  </si>
-  <si>
-    <t>2405BTNNDdieutracobandatdai_240723duthaoNDpttg(1).docx</t>
-  </si>
-  <si>
-    <t>NĐ98.2024nhachungcu.docx</t>
-  </si>
-  <si>
-    <t>NDchitietbatdongsan30.7.docx</t>
-  </si>
-  <si>
-    <t>NĐqđctmộtsốđiềuLuậtNhàở.docx</t>
-  </si>
-  <si>
-    <t>94-nd.signed.pdf</t>
-  </si>
-  <si>
-    <t>87-2025-nd-cp.signed.pdf</t>
-  </si>
-  <si>
     <t>88nd.signed.pdf</t>
   </si>
   <si>
-    <t>71-cp.signed.pdf</t>
-  </si>
-  <si>
     <t>10_2023_ND-CP.doc</t>
   </si>
   <si>
@@ -387,9 +336,6 @@
     <t>VanBanGoc_96.signed.pdf</t>
   </si>
   <si>
-    <t>12.2024.QĐ-TTg.docx</t>
-  </si>
-  <si>
     <t>VanBanGoc_48-2024-TT-BTNMT.pdf</t>
   </si>
   <si>
@@ -421,12 +367,6 @@
   </si>
   <si>
     <t>VanBanGoc_82.pdf</t>
-  </si>
-  <si>
-    <t>DUTHAOTHONGTU(bảnphathanh31.7).docx</t>
-  </si>
-  <si>
-    <t>BảntrìnhdựthảoThôngtư(final).docx</t>
   </si>
   <si>
     <t>56.2024.TT.BCA.doc</t>
@@ -721,10 +661,98 @@
 KINH DOANH BẤT ĐỘNG SẢN</t>
   </si>
   <si>
-    <t>VanBanGoc_2024_987 + 988_43-2024-QH15.pdf</t>
-  </si>
-  <si>
     <t>so_hieu</t>
+  </si>
+  <si>
+    <t>NGHỊ ĐỊNH
+Quy định việc sắp xếp lại, xử lý tài sản công là nhà, đất</t>
+  </si>
+  <si>
+    <t>VanBanGoc_2024_987.pdf</t>
+  </si>
+  <si>
+    <t>NĐ100.2024.NĐ.CP.pdf</t>
+  </si>
+  <si>
+    <t>98-2024-NĐ-CP.pdf</t>
+  </si>
+  <si>
+    <t>12-2024-QĐ-TTg.pdf</t>
+  </si>
+  <si>
+    <t>140-2025-NĐ-CP.pdf</t>
+  </si>
+  <si>
+    <t>178.2025.NĐ-CP.pdf</t>
+  </si>
+  <si>
+    <t>Nghịđịnh-192-2025-NĐ-CP.pdf</t>
+  </si>
+  <si>
+    <t>258-2025-NĐ-CP.pdf</t>
+  </si>
+  <si>
+    <t>09_2025_TT-BXD.pdf</t>
+  </si>
+  <si>
+    <t>05-2024-TT-BXD.pdf</t>
+  </si>
+  <si>
+    <t>101-2024-NĐ-CP_1.pdf</t>
+  </si>
+  <si>
+    <t>101-2024-NĐ-CP_2.pdf</t>
+  </si>
+  <si>
+    <t>115.2024.NĐ.CP_1.pdf</t>
+  </si>
+  <si>
+    <t>115.2024.NĐ.CP_2.pdf</t>
+  </si>
+  <si>
+    <t>95-2024-NĐ-CP_1.pdf</t>
+  </si>
+  <si>
+    <t>95-2024-NĐ-CP_2.pdf</t>
+  </si>
+  <si>
+    <t>95-2024-NĐ-CP_3.pdf</t>
+  </si>
+  <si>
+    <t>96-2024-NĐ-CP_1.pdf</t>
+  </si>
+  <si>
+    <t>96-2024-NĐ-CP_2.pdf</t>
+  </si>
+  <si>
+    <t>96-2024-NĐ-CP_3.pdf</t>
+  </si>
+  <si>
+    <t>96-2024-NĐ-CP_4.pdf</t>
+  </si>
+  <si>
+    <t>File 4</t>
+  </si>
+  <si>
+    <t>Nghị định-151-2025-NĐ-CP.pdf</t>
+  </si>
+  <si>
+    <t>75-2025-NĐ-CP.pdf</t>
+  </si>
+  <si>
+    <t>87-2025-nd-cp.pdf</t>
+  </si>
+  <si>
+    <t>94-nd.pdf</t>
+  </si>
+  <si>
+    <t>VanBanGoc_103-nd_1.pdf</t>
+  </si>
+  <si>
+    <t>VanBanGoc_103-nd_2.pdf</t>
+  </si>
+  <si>
+    <t>108-2024-NĐ-CP.pdf</t>
   </si>
 </sst>
 </file>
@@ -1136,25 +1164,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED14D7C1-14A4-44A5-A6EE-F18154C6E1E7}">
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28" style="9" customWidth="1"/>
-    <col min="4" max="4" width="29.5546875" style="3" customWidth="1"/>
-    <col min="5" max="6" width="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>197</v>
+        <v>176</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>65</v>
@@ -1165,13 +1195,16 @@
       <c r="F1" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="C2" s="7">
         <v>45309</v>
@@ -1186,12 +1219,12 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>194</v>
+        <v>174</v>
       </c>
       <c r="C3" s="7">
         <v>42332</v>
@@ -1203,12 +1236,12 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="C4" s="7">
         <v>37951</v>
@@ -1217,26 +1250,26 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="C5" s="7">
         <v>45472</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>136</v>
+        <v>116</v>
       </c>
       <c r="C6" s="7">
         <v>43999</v>
@@ -1248,12 +1281,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="C7" s="7">
         <v>45258</v>
@@ -1262,12 +1295,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="C8" s="7">
         <v>45625</v>
@@ -1276,12 +1309,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="C9" s="7">
         <v>43063</v>
@@ -1290,12 +1323,12 @@
         <v>73</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>139</v>
+        <v>119</v>
       </c>
       <c r="C10" s="7">
         <v>43999</v>
@@ -1304,12 +1337,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="C11" s="7">
         <v>45625</v>
@@ -1318,12 +1351,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="C12" s="7">
         <v>45833</v>
@@ -1332,12 +1365,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="C13" s="7">
         <v>43629</v>
@@ -1346,12 +1379,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="C14" s="7">
         <v>41809</v>
@@ -1360,12 +1393,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="C15" s="7">
         <v>45257</v>
@@ -1377,12 +1410,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="C16" s="7">
         <v>40348</v>
@@ -1396,7 +1429,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
       <c r="C17" s="7">
         <v>36515</v>
@@ -1410,7 +1443,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
       <c r="C18" s="7">
         <v>45940</v>
@@ -1424,13 +1457,13 @@
         <v>17</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
       <c r="C19" s="7">
         <v>45939</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>84</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1438,13 +1471,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>149</v>
+        <v>129</v>
       </c>
       <c r="C20" s="8">
         <v>45888</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -1452,13 +1485,13 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C21" s="7">
         <v>45884</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
@@ -1466,13 +1499,13 @@
         <v>20</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
       <c r="C22" s="7">
         <v>45839</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>87</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="144" x14ac:dyDescent="0.3">
@@ -1480,13 +1513,13 @@
         <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="C23" s="7">
         <v>45748</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>88</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1494,16 +1527,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>153</v>
+        <v>133</v>
       </c>
       <c r="C24" s="7">
         <v>45470</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E24" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1511,13 +1544,13 @@
         <v>23</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>154</v>
+        <v>134</v>
       </c>
       <c r="C25" s="7">
         <v>45820</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>91</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1525,13 +1558,13 @@
         <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>155</v>
+        <v>135</v>
       </c>
       <c r="C26" s="7">
         <v>45820</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1539,27 +1572,27 @@
         <v>25</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="C27" s="7">
         <v>45820</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="C28" s="8">
         <v>45658</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -1567,13 +1600,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="C29" s="8">
         <v>45839</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>95</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1581,13 +1614,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
       <c r="C30" s="8">
         <v>45820</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>96</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1595,13 +1628,13 @@
         <v>29</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
       <c r="C31" s="7">
         <v>45569</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1609,461 +1642,471 @@
         <v>30</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="C32" s="7">
         <v>45551</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+      <c r="E32" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="C33" s="7">
         <v>45527</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>162</v>
+        <v>142</v>
       </c>
       <c r="C34" s="7">
         <v>45504</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>163</v>
+        <v>143</v>
       </c>
       <c r="C35" s="7">
         <v>45503</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>164</v>
+        <v>144</v>
       </c>
       <c r="C36" s="7">
         <v>45503</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="C37" s="7">
         <v>45502</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>188</v>
+      </c>
+      <c r="E37" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>166</v>
+        <v>146</v>
       </c>
       <c r="C38" s="7">
         <v>45499</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="C39" s="7">
         <v>45498</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>168</v>
+        <v>148</v>
       </c>
       <c r="C40" s="7">
         <v>45497</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+      <c r="E40" t="s">
+        <v>196</v>
+      </c>
+      <c r="F40" t="s">
+        <v>197</v>
+      </c>
+      <c r="G40" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
       <c r="C41" s="7">
         <v>45257</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+      <c r="E41" t="s">
+        <v>193</v>
+      </c>
+      <c r="F41" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="C42" s="7">
         <v>45497</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="C43" s="7">
         <v>45758</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="C44" s="7">
         <v>45488</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>153</v>
       </c>
       <c r="C45" s="7">
-        <v>45470</v>
+        <v>45019</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="C46" s="7">
-        <v>45019</v>
+        <v>44741</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="C47" s="7">
-        <v>44741</v>
+        <v>43818</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="C48" s="7">
-        <v>43818</v>
+        <v>45504</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="C49" s="7">
-        <v>45504</v>
+        <v>45657</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="C50" s="7">
         <v>45657</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>178</v>
+        <v>159</v>
       </c>
       <c r="C51" s="7">
-        <v>45657</v>
+        <v>45638</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="C52" s="7">
-        <v>45638</v>
+        <v>45583</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>181</v>
+        <v>162</v>
       </c>
       <c r="C53" s="7">
-        <v>45583</v>
+        <v>45504</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>182</v>
+        <v>163</v>
       </c>
       <c r="C54" s="7">
         <v>45504</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>52</v>
+        <v>104</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>183</v>
+        <v>164</v>
       </c>
       <c r="C55" s="7">
-        <v>45504</v>
+        <v>45828</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>122</v>
+        <v>53</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="C56" s="7">
         <v>45828</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C57" s="7">
-        <v>45828</v>
+        <v>166</v>
+      </c>
+      <c r="C57" s="8">
+        <v>38444</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="C58" s="8">
-        <v>38444</v>
+        <v>167</v>
+      </c>
+      <c r="C58" s="7">
+        <v>45503</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B59" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C59" s="7">
+        <v>45621</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C60" s="7">
+        <v>45504</v>
+      </c>
+      <c r="D60" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="C59" s="7">
-        <v>45503</v>
-      </c>
-      <c r="D59" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A60" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="C60" s="7">
-        <v>45621</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="61" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>189</v>
+        <v>170</v>
       </c>
       <c r="C61" s="7">
-        <v>45504</v>
+        <v>45821</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>190</v>
+        <v>171</v>
       </c>
       <c r="C62" s="7">
-        <v>45821</v>
+        <v>45601</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>59</v>
+        <v>110</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>191</v>
+        <v>172</v>
       </c>
       <c r="C63" s="7">
-        <v>45601</v>
+        <v>45607</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A64" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="C64" s="7">
-        <v>45607</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: fix for Luat Dan Su
</commit_message>
<xml_diff>
--- a/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
+++ b/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\LawAssistant\triplet_extraction\data\luat_dat_dai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D44C7A7-D740-4373-AAD7-F7034A93D00D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA50280A-3A23-4896-994A-7B68408E8840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75A87B30-D479-4520-B3E8-6EE7229C7E16}"/>
   </bookViews>
@@ -591,9 +591,6 @@
 Quy định kỹ thuật về lập, điều chỉnh quy hoạch, kế hoạch sử dụng đất </t>
   </si>
   <si>
-    <t>TT29-2024-TT-BTNMT_Signed-quyđịnhkỹthuậtlập.doc</t>
-  </si>
-  <si>
     <t>THÔNG TƯ
 Quy định về việc lập, quản lý hồ sơ địa giới đơn vị hành chính</t>
   </si>
@@ -753,6 +750,9 @@
   </si>
   <si>
     <t>108-2024-NĐ-CP.pdf</t>
+  </si>
+  <si>
+    <t>29-btnmt.pdf</t>
   </si>
 </sst>
 </file>
@@ -1178,13 +1178,13 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>112</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>65</v>
@@ -1196,7 +1196,7 @@
         <v>67</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -1224,7 +1224,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C3" s="7">
         <v>42332</v>
@@ -1261,7 +1261,7 @@
         <v>45472</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1286,7 +1286,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C7" s="7">
         <v>45258</v>
@@ -1463,7 +1463,7 @@
         <v>45939</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1505,7 +1505,7 @@
         <v>45839</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="144" x14ac:dyDescent="0.3">
@@ -1519,7 +1519,7 @@
         <v>45748</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1550,7 +1550,7 @@
         <v>45820</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1586,7 +1586,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C28" s="8">
         <v>45658</v>
@@ -1606,7 +1606,7 @@
         <v>45839</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1620,7 +1620,7 @@
         <v>45820</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1648,10 +1648,10 @@
         <v>45551</v>
       </c>
       <c r="D32" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E32" t="s">
         <v>190</v>
-      </c>
-      <c r="E32" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1665,7 +1665,7 @@
         <v>45527</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1693,10 +1693,10 @@
         <v>45503</v>
       </c>
       <c r="D35" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="E35" s="3" t="s">
         <v>204</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1724,10 +1724,10 @@
         <v>45502</v>
       </c>
       <c r="D37" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="E37" t="s">
         <v>188</v>
-      </c>
-      <c r="E37" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1741,7 +1741,7 @@
         <v>45499</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1755,7 +1755,7 @@
         <v>45498</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1769,16 +1769,16 @@
         <v>45497</v>
       </c>
       <c r="D40" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="E40" t="s">
         <v>195</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
         <v>196</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>197</v>
-      </c>
-      <c r="G40" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1792,13 +1792,13 @@
         <v>45257</v>
       </c>
       <c r="D41" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E41" t="s">
         <v>192</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>193</v>
-      </c>
-      <c r="F41" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1812,7 +1812,7 @@
         <v>45497</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1826,7 +1826,7 @@
         <v>45758</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1896,7 +1896,7 @@
         <v>45504</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
@@ -1938,7 +1938,7 @@
         <v>45638</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>160</v>
+        <v>206</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -1946,7 +1946,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C52" s="7">
         <v>45583</v>
@@ -1960,7 +1960,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C53" s="7">
         <v>45504</v>
@@ -1974,7 +1974,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C54" s="7">
         <v>45504</v>
@@ -1988,7 +1988,7 @@
         <v>104</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C55" s="7">
         <v>45828</v>
@@ -2002,7 +2002,7 @@
         <v>53</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C56" s="7">
         <v>45828</v>
@@ -2016,7 +2016,7 @@
         <v>54</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C57" s="8">
         <v>38444</v>
@@ -2030,7 +2030,7 @@
         <v>55</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C58" s="7">
         <v>45503</v>
@@ -2044,7 +2044,7 @@
         <v>56</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C59" s="7">
         <v>45621</v>
@@ -2058,13 +2058,13 @@
         <v>57</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C60" s="7">
         <v>45504</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
@@ -2072,13 +2072,13 @@
         <v>58</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C61" s="7">
         <v>45821</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
@@ -2086,7 +2086,7 @@
         <v>59</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C62" s="7">
         <v>45601</v>
@@ -2100,7 +2100,7 @@
         <v>110</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C63" s="7">
         <v>45607</v>

</xml_diff>

<commit_message>
feat: improvement to data
</commit_message>
<xml_diff>
--- a/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
+++ b/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\LawAssistant\triplet_extraction\data\luat_dat_dai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA50280A-3A23-4896-994A-7B68408E8840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3C2609-792F-4EB7-B451-A116B5555D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75A87B30-D479-4520-B3E8-6EE7229C7E16}"/>
   </bookViews>
@@ -348,9 +348,6 @@
     <t>VanBanGoc_56.pdf</t>
   </si>
   <si>
-    <t>10-btnmt.pdf</t>
-  </si>
-  <si>
     <t>23-bnnmt.pdf</t>
   </si>
   <si>
@@ -753,6 +750,9 @@
   </si>
   <si>
     <t>29-btnmt.pdf</t>
+  </si>
+  <si>
+    <t>10_2024_TT-BTNMT_608554.doc</t>
   </si>
 </sst>
 </file>
@@ -1178,13 +1178,13 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>65</v>
@@ -1196,7 +1196,7 @@
         <v>67</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -1204,7 +1204,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C2" s="7">
         <v>45309</v>
@@ -1224,7 +1224,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C3" s="7">
         <v>42332</v>
@@ -1241,7 +1241,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C4" s="7">
         <v>37951</v>
@@ -1255,13 +1255,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C5" s="7">
         <v>45472</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1269,7 +1269,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C6" s="7">
         <v>43999</v>
@@ -1286,7 +1286,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7" s="7">
         <v>45258</v>
@@ -1300,7 +1300,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C8" s="7">
         <v>45625</v>
@@ -1314,7 +1314,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C9" s="7">
         <v>43063</v>
@@ -1328,7 +1328,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C10" s="7">
         <v>43999</v>
@@ -1342,7 +1342,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C11" s="7">
         <v>45625</v>
@@ -1356,7 +1356,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C12" s="7">
         <v>45833</v>
@@ -1370,7 +1370,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C13" s="7">
         <v>43629</v>
@@ -1384,7 +1384,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C14" s="7">
         <v>41809</v>
@@ -1398,7 +1398,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C15" s="7">
         <v>45257</v>
@@ -1415,7 +1415,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C16" s="7">
         <v>40348</v>
@@ -1429,7 +1429,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C17" s="7">
         <v>36515</v>
@@ -1443,7 +1443,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C18" s="7">
         <v>45940</v>
@@ -1457,13 +1457,13 @@
         <v>17</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C19" s="7">
         <v>45939</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1471,7 +1471,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C20" s="8">
         <v>45888</v>
@@ -1485,7 +1485,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C21" s="7">
         <v>45884</v>
@@ -1499,13 +1499,13 @@
         <v>20</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C22" s="7">
         <v>45839</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="144" x14ac:dyDescent="0.3">
@@ -1513,13 +1513,13 @@
         <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C23" s="7">
         <v>45748</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1527,7 +1527,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C24" s="7">
         <v>45470</v>
@@ -1544,13 +1544,13 @@
         <v>23</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C25" s="7">
         <v>45820</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1558,7 +1558,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C26" s="7">
         <v>45820</v>
@@ -1572,7 +1572,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C27" s="7">
         <v>45820</v>
@@ -1586,7 +1586,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C28" s="8">
         <v>45658</v>
@@ -1600,13 +1600,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C29" s="8">
         <v>45839</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1614,13 +1614,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C30" s="8">
         <v>45820</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1628,7 +1628,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C31" s="7">
         <v>45569</v>
@@ -1642,16 +1642,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C32" s="7">
         <v>45551</v>
       </c>
       <c r="D32" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="E32" t="s">
         <v>189</v>
-      </c>
-      <c r="E32" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1659,13 +1659,13 @@
         <v>31</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C33" s="7">
         <v>45527</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1673,7 +1673,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C34" s="7">
         <v>45504</v>
@@ -1687,16 +1687,16 @@
         <v>33</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C35" s="7">
         <v>45503</v>
       </c>
       <c r="D35" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="E35" s="3" t="s">
         <v>203</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1704,7 +1704,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C36" s="7">
         <v>45503</v>
@@ -1718,16 +1718,16 @@
         <v>35</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C37" s="7">
         <v>45502</v>
       </c>
       <c r="D37" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E37" t="s">
         <v>187</v>
-      </c>
-      <c r="E37" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1735,13 +1735,13 @@
         <v>36</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C38" s="7">
         <v>45499</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1749,13 +1749,13 @@
         <v>37</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C39" s="7">
         <v>45498</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1763,22 +1763,22 @@
         <v>38</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C40" s="7">
         <v>45497</v>
       </c>
       <c r="D40" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E40" t="s">
         <v>194</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
         <v>195</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>196</v>
-      </c>
-      <c r="G40" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1786,19 +1786,19 @@
         <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C41" s="7">
         <v>45257</v>
       </c>
       <c r="D41" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E41" t="s">
         <v>191</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>192</v>
-      </c>
-      <c r="F41" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1806,13 +1806,13 @@
         <v>40</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C42" s="7">
         <v>45497</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1820,13 +1820,13 @@
         <v>41</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C43" s="7">
         <v>45758</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1834,7 +1834,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C44" s="7">
         <v>45488</v>
@@ -1848,7 +1848,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C45" s="7">
         <v>45019</v>
@@ -1862,7 +1862,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C46" s="7">
         <v>44741</v>
@@ -1876,7 +1876,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C47" s="7">
         <v>43818</v>
@@ -1890,13 +1890,13 @@
         <v>46</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C48" s="7">
         <v>45504</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
@@ -1904,7 +1904,7 @@
         <v>47</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C49" s="7">
         <v>45657</v>
@@ -1918,7 +1918,7 @@
         <v>48</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C50" s="7">
         <v>45657</v>
@@ -1932,13 +1932,13 @@
         <v>49</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C51" s="7">
         <v>45638</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -1946,7 +1946,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C52" s="7">
         <v>45583</v>
@@ -1960,7 +1960,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C53" s="7">
         <v>45504</v>
@@ -1974,27 +1974,27 @@
         <v>52</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C54" s="7">
         <v>45504</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>102</v>
+        <v>206</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C55" s="7">
         <v>45828</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
@@ -2002,13 +2002,13 @@
         <v>53</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C56" s="7">
         <v>45828</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
@@ -2016,13 +2016,13 @@
         <v>54</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C57" s="8">
         <v>38444</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
@@ -2030,13 +2030,13 @@
         <v>55</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C58" s="7">
         <v>45503</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
@@ -2044,13 +2044,13 @@
         <v>56</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C59" s="7">
         <v>45621</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -2058,13 +2058,13 @@
         <v>57</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C60" s="7">
         <v>45504</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
@@ -2072,13 +2072,13 @@
         <v>58</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C61" s="7">
         <v>45821</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
@@ -2086,27 +2086,27 @@
         <v>59</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C62" s="7">
         <v>45601</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C63" s="7">
         <v>45607</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add "Tieu muc"
</commit_message>
<xml_diff>
--- a/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
+++ b/triplet_extraction/data/luat_dat_dai/Luat_dat_dai_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\LawAssistant\triplet_extraction\data\luat_dat_dai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3C2609-792F-4EB7-B451-A116B5555D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DF1F9A8-7E83-498D-AD95-E7FE1E6698D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{75A87B30-D479-4520-B3E8-6EE7229C7E16}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
   <si>
     <t>31/2024/QH15</t>
   </si>
@@ -183,12 +183,6 @@
     <t>12/2024/QĐ-TTg</t>
   </si>
   <si>
-    <t>48/2024/TT-BTNMT</t>
-  </si>
-  <si>
-    <t>50/2024/TT-BTNMT</t>
-  </si>
-  <si>
     <t>29/2024/TT-BTNMT</t>
   </si>
   <si>
@@ -334,12 +328,6 @@
   </si>
   <si>
     <t>VanBanGoc_96.signed.pdf</t>
-  </si>
-  <si>
-    <t>VanBanGoc_48-2024-TT-BTNMT.pdf</t>
-  </si>
-  <si>
-    <t>50-btnmt.pdf</t>
   </si>
   <si>
     <t>11-bnv.pdf</t>
@@ -571,17 +559,6 @@
   <si>
     <t>QUYẾT ĐỊNH
 VỀ CƠ CHẾ, CHÍNH SÁCH GIẢI QUYẾT VIỆC LÀM VÀ ĐÀO TẠO NGHỀ CHO NGƯỜI CÓ ĐẤT THU HỒI</t>
-  </si>
-  <si>
-    <t>THÔNG TƯ
-Quy định định mức kinh tế - kỹ thuật
-thống kê, kiểm kê đất đai, lập bản đồ hiện trạng sử dụng đất và xây dựng
-cơ sở dữ liệu quốc gia về đất đai</t>
-  </si>
-  <si>
-    <t>THÔNG TƯ
-Quy định định mức kinh tế - kỹ thuật điều tra, đánh giá đất đai
-cấp vùng và cả nước</t>
   </si>
   <si>
     <t xml:space="preserve">THÔNG TƯ
@@ -1164,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED14D7C1-14A4-44A5-A6EE-F18154C6E1E7}">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" style="2" bestFit="1" customWidth="1"/>
@@ -1178,25 +1155,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -1204,19 +1181,19 @@
         <v>0</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C2" s="7">
         <v>45309</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" t="s">
         <v>60</v>
-      </c>
-      <c r="E2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -1224,16 +1201,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C3" s="7">
         <v>42332</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
@@ -1241,13 +1218,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C4" s="7">
         <v>37951</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
@@ -1255,13 +1232,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C5" s="7">
         <v>45472</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1269,16 +1246,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C6" s="7">
         <v>43999</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1286,13 +1263,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C7" s="7">
         <v>45258</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1300,13 +1277,13 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C8" s="7">
         <v>45625</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1314,13 +1291,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C9" s="7">
         <v>43063</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -1328,13 +1305,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C10" s="7">
         <v>43999</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1342,13 +1319,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C11" s="7">
         <v>45625</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
@@ -1356,13 +1333,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C12" s="7">
         <v>45833</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -1370,13 +1347,13 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C13" s="7">
         <v>43629</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1384,13 +1361,13 @@
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C14" s="7">
         <v>41809</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1398,16 +1375,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C15" s="7">
         <v>45257</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1415,13 +1392,13 @@
         <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C16" s="7">
         <v>40348</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1429,13 +1406,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C17" s="7">
         <v>36515</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="216" x14ac:dyDescent="0.3">
@@ -1443,13 +1420,13 @@
         <v>16</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C18" s="7">
         <v>45940</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1457,13 +1434,13 @@
         <v>17</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C19" s="7">
         <v>45939</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1471,13 +1448,13 @@
         <v>18</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C20" s="8">
         <v>45888</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -1485,13 +1462,13 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C21" s="7">
         <v>45884</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
@@ -1499,13 +1476,13 @@
         <v>20</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C22" s="7">
         <v>45839</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="144" x14ac:dyDescent="0.3">
@@ -1513,13 +1490,13 @@
         <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C23" s="7">
         <v>45748</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1527,16 +1504,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C24" s="7">
         <v>45470</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E24" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1544,13 +1521,13 @@
         <v>23</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C25" s="7">
         <v>45820</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1558,13 +1535,13 @@
         <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C26" s="7">
         <v>45820</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1572,13 +1549,13 @@
         <v>25</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C27" s="7">
         <v>45820</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1586,13 +1563,13 @@
         <v>26</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C28" s="8">
         <v>45658</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
@@ -1600,13 +1577,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C29" s="8">
         <v>45839</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
@@ -1614,13 +1591,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C30" s="8">
         <v>45820</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
@@ -1628,13 +1605,13 @@
         <v>29</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C31" s="7">
         <v>45569</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="72" x14ac:dyDescent="0.3">
@@ -1642,16 +1619,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C32" s="7">
         <v>45551</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="E32" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1659,13 +1636,13 @@
         <v>31</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C33" s="7">
         <v>45527</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1673,13 +1650,13 @@
         <v>32</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C34" s="7">
         <v>45504</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1687,16 +1664,16 @@
         <v>33</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C35" s="7">
         <v>45503</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1704,13 +1681,13 @@
         <v>34</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C36" s="7">
         <v>45503</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
@@ -1718,16 +1695,16 @@
         <v>35</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C37" s="7">
         <v>45502</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="E37" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1735,13 +1712,13 @@
         <v>36</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C38" s="7">
         <v>45499</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1749,13 +1726,13 @@
         <v>37</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C39" s="7">
         <v>45498</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1763,22 +1740,22 @@
         <v>38</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C40" s="7">
         <v>45497</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="E40" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="F40" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="G40" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1786,19 +1763,19 @@
         <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C41" s="7">
         <v>45257</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E41" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="F41" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1806,13 +1783,13 @@
         <v>40</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C42" s="7">
         <v>45497</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1820,13 +1797,13 @@
         <v>41</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C43" s="7">
         <v>45758</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -1834,13 +1811,13 @@
         <v>42</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C44" s="7">
         <v>45488</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -1848,13 +1825,13 @@
         <v>43</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C45" s="7">
         <v>45019</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1862,13 +1839,13 @@
         <v>44</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C46" s="7">
         <v>44741</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -1876,13 +1853,13 @@
         <v>45</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C47" s="7">
         <v>43818</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1890,223 +1867,195 @@
         <v>46</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C48" s="7">
         <v>45504</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C49" s="7">
-        <v>45657</v>
+        <v>45638</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C50" s="7">
-        <v>45657</v>
+        <v>45583</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C51" s="7">
-        <v>45638</v>
+        <v>45504</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C52" s="7">
-        <v>45583</v>
+        <v>45504</v>
       </c>
       <c r="D52" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C53" s="7">
+        <v>45828</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C54" s="7">
+        <v>45828</v>
+      </c>
+      <c r="D54" s="3" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A53" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="C53" s="7">
-        <v>45504</v>
-      </c>
-      <c r="D53" s="3" t="s">
+    <row r="55" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C55" s="8">
+        <v>38444</v>
+      </c>
+      <c r="D55" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A54" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="C54" s="7">
-        <v>45504</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="C55" s="7">
-        <v>45828</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C56" s="7">
-        <v>45828</v>
+        <v>45503</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="C57" s="8">
-        <v>38444</v>
+        <v>160</v>
+      </c>
+      <c r="C57" s="7">
+        <v>45621</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C58" s="7">
-        <v>45503</v>
+        <v>45504</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C59" s="7">
-        <v>45621</v>
+        <v>45821</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C60" s="7">
-        <v>45504</v>
+        <v>45601</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C61" s="7">
-        <v>45821</v>
+        <v>45607</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A62" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="C62" s="7">
-        <v>45601</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="C63" s="7">
-        <v>45607</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>